<commit_message>
Kijk de zeven recordvragen na en corrigeer er drie
Ze droegen de markering "veroudert" omdat records gebroken worden. Bij drie
verhulde die markering iets anders: het antwoord was gewoon fout. Het aantal
marathons van Horst Preisler is 1305 en niet 1000, het jongleerrecord van
Edinburgh 1508 en niet 1000, en de langste gamemarathon staat op 144 uur.

Bij twee was "veroudert" juist onnodig: de hoogste klifduik staat sinds 2015 en
het push-uprecord sinds 1993. Die zijn nu als bevestigd gemarkeerd.

Zeven puzzels breken hierdoor; ze staan in het herbouwoverzicht.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vragen/1000+ vragen netjes gecategoriseerd.xlsx
+++ b/vragen/1000+ vragen netjes gecategoriseerd.xlsx
@@ -9307,11 +9307,11 @@
         </is>
       </c>
       <c r="C444" t="n">
-        <v>1000</v>
+        <v>1305</v>
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>https://www.guinnessworldrecords.com/world-records/most-marathons-run</t>
+          <t>https://www.guinnessworldrecords.com/world-records/64777-most-marathons-completed</t>
         </is>
       </c>
     </row>
@@ -9383,15 +9383,15 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>Hoeveel uur duurde het langste videogame-marathonrecord?</t>
+          <t>Hoeveel uur duurde het langste videogame-marathonrecord (stand 2026)?</t>
         </is>
       </c>
       <c r="C448" t="n">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>https://www.guinnessworldrecords.com/world-records/longest-videogames-marathon</t>
+          <t>https://www.guinnessworldrecords.com/world-records/longest-video-games-marathon</t>
         </is>
       </c>
     </row>
@@ -26366,7 +26366,7 @@
       </c>
       <c r="D1204" t="inlineStr">
         <is>
-          <t>https://www.guinnessworldrecords.com/world-records/highest-dive</t>
+          <t>https://www.guinnessworldrecords.com/world-records/407825-highest-cliff-jump</t>
         </is>
       </c>
     </row>
@@ -26642,11 +26642,11 @@
         </is>
       </c>
       <c r="C1218" t="n">
-        <v>1000</v>
+        <v>1508</v>
       </c>
       <c r="D1218" t="inlineStr">
         <is>
-          <t>https://www.guinnessworldrecords.com/</t>
+          <t>https://www.guinnessworldrecords.com/world-records/68643-most-people-juggling-simultaneously</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Vervang negen bronnen die naar de verkeerde pagina wezen
De eerdere screening keek of het adres nog enig woord uit de vraag bevatte. Dat
mist het geval waarin dat woord er wel in staat maar de pagina toch verkeerd is:
de wielen van een Boeing 747 wezen naar het artikel over het bedrijf Boeing, met
als bewijs dat de 737 MAX 18 miljard dollar kostte.

Deze ronde toetst of het antwoord überhaupt in de bewijszin staat. Bij 22 van de
662 bronnen met vertrouwen hoog niet. Negen bleken een echt verkeerde pagina,
waaronder drie doorverwijspagina's: Chili wees naar chilipeper, Mars naar het
woord Mars, en de Chinese dierenriem naar schorpioenen.

De overige dertien houden hun bron en krijgen een bewijszin die wel iets zegt.
Antwoorden onveranderd, dus geen puzzel breekt.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vragen/1000+ vragen netjes gecategoriseerd.xlsx
+++ b/vragen/1000+ vragen netjes gecategoriseerd.xlsx
@@ -3211,7 +3211,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://nl.wikipedia.org/wiki/Mars</t>
+          <t>https://nl.wikipedia.org/wiki/Mars_(planeet)</t>
         </is>
       </c>
     </row>
@@ -6211,7 +6211,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/HC_Klein_Zwitserland</t>
+          <t>https://nl.wikipedia.org/wiki/Zwitserland</t>
         </is>
       </c>
     </row>
@@ -7331,7 +7331,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/UNESCO</t>
+          <t>https://ich.unesco.org/en/intangible-heritage-domains-00052</t>
         </is>
       </c>
     </row>
@@ -8071,7 +8071,7 @@
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>https://nl.wikipedia.org/wiki/Bad_Bunny</t>
+          <t>https://en.wikipedia.org/wiki/Un_Verano_Sin_Ti</t>
         </is>
       </c>
     </row>
@@ -11936,7 +11936,7 @@
       </c>
       <c r="D575" t="inlineStr">
         <is>
-          <t>https://nl.wikipedia.org/wiki/Boeing</t>
+          <t>https://nl.wikipedia.org/wiki/Boeing_747</t>
         </is>
       </c>
     </row>
@@ -13741,7 +13741,7 @@
       </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>https://nl.wikipedia.org/wiki/Schorpioenen_%28dieren%29</t>
+          <t>https://nl.wikipedia.org/wiki/Chinese_astrologie</t>
         </is>
       </c>
       <c r="E659" t="inlineStr">
@@ -17691,7 +17691,7 @@
       </c>
       <c r="D832" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Chili</t>
+          <t>https://en.wikipedia.org/wiki/Chile</t>
         </is>
       </c>
       <c r="E832" t="inlineStr">
@@ -23731,7 +23731,7 @@
       </c>
       <c r="D1094" t="inlineStr">
         <is>
-          <t>https://nl.wikipedia.org/wiki/Utrecht_%28stad%29</t>
+          <t>https://nl.wikipedia.org/wiki/Nederlands_Film_Festival</t>
         </is>
       </c>
       <c r="E1094" t="inlineStr">
@@ -27401,7 +27401,7 @@
       </c>
       <c r="D1254" t="inlineStr">
         <is>
-          <t>https://nl.wikipedia.org/wiki/Olympische_Zomerspelen</t>
+          <t>https://nl.wikipedia.org/wiki/Olympische_Zomerspelen_2024</t>
         </is>
       </c>
       <c r="E1254" t="inlineStr">

</xml_diff>